<commit_message>
Liste ve plan dosyası yenilendi — 11-19 Ekim, 9 gün
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DAKoXHyqFjWGSzqcjwTyja
</commit_message>
<xml_diff>
--- a/yayin-plani.xlsx
+++ b/yayin-plani.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$L$82</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$L$84</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="155">
   <si>
     <t xml:space="preserve">YAYIN PLANI · 11-18 Ekim 2026</t>
   </si>
@@ -230,211 +230,217 @@
     <t xml:space="preserve">2026-10-16-sunlu-filament-pano</t>
   </si>
   <si>
+    <t xml:space="preserve">Phaetus Conch M4 Endcoat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13-phaetus-conch-nozul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunlu AMS Heater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-sunlu-ams-heater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prototip Çalıştı Ürün Tutmuyor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13-olcu-dogrulama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Çarşamba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,4 Her İşe Yetiyor Mu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13-nozzle-capi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BMS Neyi Koruyor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14-lipo-bms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phaetus × Snapmaker Liber Hotend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16-phaetus-liber-u1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siparişi Kabul Etmeden Önce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14-siparis-sorulari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perşembe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi Kurutucu Sana Uygun?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-filament-kurutucu-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayrık H Köprüsü Mü, DRV8833 Mü</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-h-koprusu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polymaker HT-PLA Serisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-17-polymaker-ht-pla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Son Gün · Dört Makara Tek Kişiye 23.59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-cekilis-son-gun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Var Olan Parçayı Tarayıp Kopyalamak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-3d-tarayici</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H Serisinde Fark Ne?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-bambu-h-serisi-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projeye Hangi Kart Girer?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16-gelistirme-karti-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atık Üretmeden Renk Değiştirmek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-21-u1-k3-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi Pixhawk Yeterli?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20-pixhawk-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumartesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Serisinde Hangisi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-19-bambu-a-serisi-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi ESP32 Senin İşine?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-17-esp32-ailesi-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparkX İ7 Mi İ8 Mi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20-sparkx-i7-i8-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi Pı Kamerası?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-21-pi-kamera-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pirinç Uç Ne Zaman Biter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-sert-nozul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kondansatör Sağlam Görünüp Bozuk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-kondansator-esr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ender-3 V4 Combo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-ender-3-v4-combo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bozuk Baskıyı Tek Başına Çözme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-toplulukta-ariza</t>
+  </si>
+  <si>
     <t xml:space="preserve">Optokuplör Ne Zaman Şart</t>
   </si>
   <si>
     <t xml:space="preserve">2026-10-13-optokuplor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sunlu AMS Heater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-sunlu-ams-heater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prototip Çalıştı Ürün Tutmuyor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-13-olcu-dogrulama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Çarşamba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,4 Her İşe Yetiyor Mu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-13-nozzle-capi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BMS Neyi Koruyor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-14-lipo-bms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phaetus × Snapmaker Liber Hotend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16-phaetus-liber-u1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siparişi Kabul Etmeden Önce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-14-siparis-sorulari</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perşembe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi Kurutucu Sana Uygun?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-filament-kurutucu-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ayrık H Köprüsü Mü, DRV8833 Mü</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-h-koprusu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polymaker HT-PLA Serisi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-17-polymaker-ht-pla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Son Gün · Dört Makara Tek Kişiye 23.59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-cekilis-son-gun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Var Olan Parçayı Tarayıp Kopyalamak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-3d-tarayici</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H Serisinde Fark Ne?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-bambu-h-serisi-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projeye Hangi Kart Girer?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16-gelistirme-karti-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atık Üretmeden Renk Değiştirmek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-21-u1-k3-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi Pixhawk Yeterli?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20-pixhawk-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cumartesi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Serisinde Hangisi?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-19-bambu-a-serisi-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi ESP32 Senin İşine?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-17-esp32-ailesi-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparkX İ7 Mi İ8 Mi?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20-sparkx-i7-i8-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi Pı Kamerası?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-21-pi-kamera-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pirinç Uç Ne Zaman Biter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-sert-nozul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kondansatör Sağlam Görünüp Bozuk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-kondansator-esr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ender-3 V4 Combo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-ender-3-v4-combo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bozuk Baskıyı Tek Başına Çözme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-toplulukta-ariza</t>
   </si>
   <si>
     <t xml:space="preserve">ÖZET</t>
@@ -1128,7 +1134,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11"/>
@@ -2024,7 +2030,7 @@
         <v>20</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>1007</v>
+        <v>0</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>21</v>
@@ -4011,12 +4017,84 @@
       </c>
       <c r="L82" s="11"/>
     </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="4" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F83" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="H83" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I83" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J83" s="9" t="n">
+        <v>1007</v>
+      </c>
+      <c r="K83" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="L83" s="5"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="4" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C84" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D84" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E84" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F84" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="G84" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="H84" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I84" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="J84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="L84" s="11"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L82"/>
+  <autoFilter ref="A4:L84"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
-  <conditionalFormatting sqref="K5:K82">
+  <conditionalFormatting sqref="K5:K84">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yayınlandı"</formula>
     </cfRule>
@@ -4025,7 +4103,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" error="Listeden seç: Bekliyor, Yayınlandı, Atlandı" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K82" type="list">
+    <dataValidation allowBlank="false" error="Listeden seç: Bekliyor, Yayınlandı, Atlandı" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K84" type="list">
       <formula1>"Bekliyor,Yayınlandı,Atlandı"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4046,7 +4124,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -4061,17 +4139,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4079,16 +4157,16 @@
         <v>5</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4096,16 +4174,16 @@
         <v>16</v>
       </c>
       <c r="B6" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$82,A6)</f>
-        <v>32</v>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A6)</f>
+        <v>33</v>
       </c>
       <c r="C6" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$82,A6,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A6,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D6" s="20" t="n">
         <f aca="false">B6-C6</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" s="21" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
@@ -4117,16 +4195,16 @@
         <v>23</v>
       </c>
       <c r="B7" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$82,A7)</f>
-        <v>36</v>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A7)</f>
+        <v>37</v>
       </c>
       <c r="C7" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$82,A7,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A7,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">B7-C7</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" s="21" t="n">
         <f aca="false">IF(B7=0,0,C7/B7)</f>
@@ -4138,11 +4216,11 @@
         <v>34</v>
       </c>
       <c r="B8" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$82,A8)</f>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A8)</f>
         <v>8</v>
       </c>
       <c r="C8" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$82,A8,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A8,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D8" s="20" t="n">
@@ -4159,11 +4237,11 @@
         <v>52</v>
       </c>
       <c r="B9" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$82,A9)</f>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A9)</f>
         <v>2</v>
       </c>
       <c r="C9" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$82,A9,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A9,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D9" s="20" t="n">
@@ -4177,11 +4255,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B10" s="26" t="n">
         <f aca="false">SUM(B6:B9)</f>
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C10" s="26" t="n">
         <f aca="false">SUM(C6:C9)</f>
@@ -4189,7 +4267,7 @@
       </c>
       <c r="D10" s="26" t="n">
         <f aca="false">SUM(D6:D9)</f>
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E10" s="27" t="n">
         <f aca="false">IF(B10=0,0,C10/B10)</f>
@@ -4198,7 +4276,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4209,25 +4287,25 @@
         <v>3</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4238,19 +4316,19 @@
         <v>14</v>
       </c>
       <c r="C15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A15,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A15,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A15,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A15,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G15" s="20" t="n">
@@ -4258,7 +4336,7 @@
         <v>9</v>
       </c>
       <c r="H15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A15,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I15" s="21" t="n">
@@ -4274,19 +4352,19 @@
         <v>42</v>
       </c>
       <c r="C16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A16,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A16,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A16,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A16,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>1</v>
       </c>
       <c r="G16" s="20" t="n">
@@ -4294,7 +4372,7 @@
         <v>11</v>
       </c>
       <c r="H16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A16,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I16" s="21" t="n">
@@ -4310,19 +4388,19 @@
         <v>65</v>
       </c>
       <c r="C17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A17,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A17,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A17,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A17,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G17" s="20" t="n">
@@ -4330,7 +4408,7 @@
         <v>10</v>
       </c>
       <c r="H17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A17,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I17" s="21" t="n">
@@ -4346,19 +4424,19 @@
         <v>78</v>
       </c>
       <c r="C18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A18,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A18,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A18,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A18,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G18" s="20" t="n">
@@ -4366,7 +4444,7 @@
         <v>10</v>
       </c>
       <c r="H18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A18,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I18" s="21" t="n">
@@ -4382,19 +4460,19 @@
         <v>87</v>
       </c>
       <c r="C19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A19,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A19,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A19,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A19,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>1</v>
       </c>
       <c r="G19" s="20" t="n">
@@ -4402,7 +4480,7 @@
         <v>11</v>
       </c>
       <c r="H19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A19,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I19" s="21" t="n">
@@ -4418,19 +4496,19 @@
         <v>100</v>
       </c>
       <c r="C20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A20,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A20,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A20,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A20,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G20" s="20" t="n">
@@ -4438,7 +4516,7 @@
         <v>9</v>
       </c>
       <c r="H20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A20,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I20" s="21" t="n">
@@ -4454,19 +4532,19 @@
         <v>114</v>
       </c>
       <c r="C21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A21,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A21,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A21,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A21,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G21" s="20" t="n">
@@ -4474,7 +4552,7 @@
         <v>9</v>
       </c>
       <c r="H21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A21,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I21" s="21" t="n">
@@ -4490,19 +4568,19 @@
         <v>14</v>
       </c>
       <c r="C22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A22,Plan!$D$5:$D$82,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A22,Plan!$D$5:$D$82,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A22,Plan!$D$5:$D$82,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A22,Plan!$D$5:$D$82,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G22" s="20" t="n">
@@ -4510,7 +4588,7 @@
         <v>9</v>
       </c>
       <c r="H22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$82,$A22,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I22" s="21" t="n">
@@ -4519,122 +4597,158 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="C23" s="26" t="n">
-        <f aca="false">SUM(C15:C22)</f>
-        <v>32</v>
-      </c>
-      <c r="D23" s="26" t="n">
-        <f aca="false">SUM(D15:D22)</f>
-        <v>36</v>
-      </c>
-      <c r="E23" s="26" t="n">
-        <f aca="false">SUM(E15:E22)</f>
+      <c r="A23" s="28" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"REELS")</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <f aca="false">SUM(C23:F23)</f>
+        <v>2</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="21" t="n">
+        <f aca="false">IF(G23=0,0,H23/G23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" s="26" t="n">
+        <f aca="false">SUM(C15:C23)</f>
+        <v>33</v>
+      </c>
+      <c r="D24" s="26" t="n">
+        <f aca="false">SUM(D15:D23)</f>
+        <v>37</v>
+      </c>
+      <c r="E24" s="26" t="n">
+        <f aca="false">SUM(E15:E23)</f>
         <v>8</v>
       </c>
-      <c r="F23" s="26" t="n">
-        <f aca="false">SUM(F15:F22)</f>
+      <c r="F24" s="26" t="n">
+        <f aca="false">SUM(F15:F23)</f>
         <v>2</v>
       </c>
-      <c r="G23" s="26" t="n">
-        <f aca="false">SUM(G15:G22)</f>
-        <v>78</v>
-      </c>
-      <c r="H23" s="26" t="n">
-        <f aca="false">SUM(H15:H22)</f>
-        <v>0</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <f aca="false">IF(G23=0,0,H23/G23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
-        <v>151</v>
+      <c r="G24" s="26" t="n">
+        <f aca="false">SUM(G15:G23)</f>
+        <v>80</v>
+      </c>
+      <c r="H24" s="26" t="n">
+        <f aca="false">SUM(H15:H23)</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <f aca="false">IF(G24=0,0,H24/G24)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="17" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$82,A28)</f>
-        <v>16</v>
-      </c>
-      <c r="C28" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$82,A28,Plan!$K$5:$K$82,"Yayınlandı")</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$82,Plan!$E$5:$E$82,A28,Plan!$D$5:$D$82,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$82,A28,Plan!$D$5:$D$82,"GÖNDERİ"),0),0)</f>
-        <v>1425</v>
+      <c r="B28" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="29" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B29" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$82,A29)</f>
+        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A29)</f>
         <v>16</v>
       </c>
       <c r="C29" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$82,A29,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A29,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D29" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$82,Plan!$E$5:$E$82,A29,Plan!$D$5:$D$82,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$82,A29,Plan!$D$5:$D$82,"GÖNDERİ"),0),0)</f>
-        <v>1314</v>
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A29,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A29,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
+        <v>1425</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="29" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B30" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$82,A30)</f>
-        <v>16</v>
+        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A30)</f>
+        <v>18</v>
       </c>
       <c r="C30" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$82,A30,Plan!$K$5:$K$82,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A30,Plan!$K$5:$K$84,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D30" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$82,Plan!$E$5:$E$82,A30,Plan!$D$5:$D$82,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$82,A30,Plan!$D$5:$D$82,"GÖNDERİ"),0),0)</f>
-        <v>1508</v>
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A30,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A30,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
+        <v>1168</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="20" t="n">
+        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A31)</f>
+        <v>16</v>
+      </c>
+      <c r="C31" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A31,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="20" t="n">
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A31,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A31,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$82,A31)</f>
+      <c r="B32" s="20" t="n">
+        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A32)</f>
         <v>16</v>
       </c>
-      <c r="C31" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$82,A31,Plan!$K$5:$K$82,"Yayınlandı")</f>
-        <v>0</v>
-      </c>
-      <c r="D31" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$82,Plan!$E$5:$E$82,A31,Plan!$D$5:$D$82,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$82,A31,Plan!$D$5:$D$82,"GÖNDERİ"),0),0)</f>
+      <c r="C32" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A32,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="20" t="n">
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A32,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A32,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
         <v>1286</v>
       </c>
     </row>

</xml_diff>

<commit_message>
13 Ekim 08:12: filament ayar rehberi — yeni tablo şablonu kuyruğa
Aynı konuyu anlatan eski pano yerine geçiyor (20 Ekim'e alındı).
Rehberdeki rakamlar kendi ürün sayfalarından; pano SUNLU föyünden
alınmış rakamlarla kendi sayfasıyla çelişiyordu, o çelişki de böylece
kalktı.

rehber.py'ye hikaye sürümü eklendi: tabloyu 9:16'ya yeniden dizmek
satırları inceltip okunmaz yapıyor, kare olduğu gibi koyu zemine
oturuyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DAKoXHyqFjWGSzqcjwTyja
</commit_message>
<xml_diff>
--- a/yayin-plani.xlsx
+++ b/yayin-plani.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$L$84</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$L$86</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="156">
   <si>
     <t xml:space="preserve">YAYIN PLANI · 11-18 Ekim 2026</t>
   </si>
@@ -224,181 +224,184 @@
     <t xml:space="preserve">Salı</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-21-filament-rehberi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phaetus Conch M4 Endcoat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13-phaetus-conch-nozul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunlu AMS Heater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-sunlu-ams-heater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prototip Çalıştı Ürün Tutmuyor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13-olcu-dogrulama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Çarşamba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,4 Her İşe Yetiyor Mu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13-nozzle-capi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BMS Neyi Koruyor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14-lipo-bms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phaetus × Snapmaker Liber Hotend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16-phaetus-liber-u1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siparişi Kabul Etmeden Önce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14-siparis-sorulari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perşembe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi Kurutucu Sana Uygun?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-filament-kurutucu-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayrık H Köprüsü Mü, DRV8833 Mü</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-h-koprusu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polymaker HT-PLA Serisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-17-polymaker-ht-pla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Son Gün · Dört Makara Tek Kişiye 23.59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-cekilis-son-gun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Var Olan Parçayı Tarayıp Kopyalamak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15-3d-tarayici</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H Serisinde Fark Ne?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18-bambu-h-serisi-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projeye Hangi Kart Girer?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16-gelistirme-karti-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atık Üretmeden Renk Değiştirmek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-21-u1-k3-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi Pixhawk Yeterli?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20-pixhawk-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumartesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Serisinde Hangisi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-19-bambu-a-serisi-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hangi ESP32 Senin İşine?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-17-esp32-ailesi-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparkX İ7 Mi İ8 Mi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20-sparkx-i7-i8-pano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hangi Sunlu Filament?</t>
   </si>
   <si>
     <t xml:space="preserve">2026-10-16-sunlu-filament-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phaetus Conch M4 Endcoat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-13-phaetus-conch-nozul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sunlu AMS Heater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-sunlu-ams-heater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prototip Çalıştı Ürün Tutmuyor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-13-olcu-dogrulama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Çarşamba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,4 Her İşe Yetiyor Mu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-13-nozzle-capi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BMS Neyi Koruyor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-14-lipo-bms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phaetus × Snapmaker Liber Hotend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16-phaetus-liber-u1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siparişi Kabul Etmeden Önce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-14-siparis-sorulari</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perşembe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi Kurutucu Sana Uygun?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-filament-kurutucu-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ayrık H Köprüsü Mü, DRV8833 Mü</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-h-koprusu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polymaker HT-PLA Serisi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-17-polymaker-ht-pla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Son Gün · Dört Makara Tek Kişiye 23.59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-cekilis-son-gun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Var Olan Parçayı Tarayıp Kopyalamak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-15-3d-tarayici</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H Serisinde Fark Ne?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-18-bambu-h-serisi-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projeye Hangi Kart Girer?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-16-gelistirme-karti-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atık Üretmeden Renk Değiştirmek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-21-u1-k3-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi Pixhawk Yeterli?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20-pixhawk-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cumartesi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Serisinde Hangisi?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-19-bambu-a-serisi-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hangi ESP32 Senin İşine?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-17-esp32-ailesi-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparkX İ7 Mi İ8 Mi?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-20-sparkx-i7-i8-pano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:30</t>
   </si>
   <si>
     <t xml:space="preserve">20:10</t>
@@ -1134,7 +1137,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11"/>
@@ -1949,7 +1952,7 @@
         <v>66</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H25" s="9" t="n">
         <v>1</v>
@@ -1958,7 +1961,7 @@
         <v>20</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>1644</v>
+        <v>0</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>21</v>
@@ -1985,7 +1988,7 @@
         <v>66</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H26" s="9" t="n">
         <v>1</v>
@@ -2018,10 +2021,10 @@
         <v>24</v>
       </c>
       <c r="F27" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="H27" s="9" t="n">
         <v>4</v>
@@ -2054,10 +2057,10 @@
         <v>24</v>
       </c>
       <c r="F28" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G28" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="H28" s="9" t="n">
         <v>1</v>
@@ -2090,10 +2093,10 @@
         <v>29</v>
       </c>
       <c r="F29" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>71</v>
       </c>
       <c r="H29" s="9" t="n">
         <v>5</v>
@@ -2126,10 +2129,10 @@
         <v>29</v>
       </c>
       <c r="F30" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G30" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="H30" s="9" t="n">
         <v>1</v>
@@ -2153,7 +2156,7 @@
         <v>65</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>23</v>
@@ -2189,7 +2192,7 @@
         <v>65</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>34</v>
@@ -2198,10 +2201,10 @@
         <v>35</v>
       </c>
       <c r="F32" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G32" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="G32" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="H32" s="9" t="n">
         <v>1</v>
@@ -2225,7 +2228,7 @@
         <v>65</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>16</v>
@@ -2234,10 +2237,10 @@
         <v>38</v>
       </c>
       <c r="F33" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G33" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>76</v>
       </c>
       <c r="H33" s="9" t="n">
         <v>4</v>
@@ -2261,7 +2264,7 @@
         <v>65</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>23</v>
@@ -2270,10 +2273,10 @@
         <v>38</v>
       </c>
       <c r="F34" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="G34" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="G34" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="H34" s="9" t="n">
         <v>1</v>
@@ -2294,7 +2297,7 @@
         <v>46309</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>43</v>
@@ -2306,10 +2309,10 @@
         <v>17</v>
       </c>
       <c r="F35" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="G35" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="H35" s="9" t="n">
         <v>4</v>
@@ -2330,7 +2333,7 @@
         <v>46309</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C36" s="10" t="s">
         <v>46</v>
@@ -2342,10 +2345,10 @@
         <v>17</v>
       </c>
       <c r="F36" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="G36" s="11" t="s">
         <v>79</v>
-      </c>
-      <c r="G36" s="11" t="s">
-        <v>80</v>
       </c>
       <c r="H36" s="9" t="n">
         <v>1</v>
@@ -2366,7 +2369,7 @@
         <v>46309</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>47</v>
@@ -2378,10 +2381,10 @@
         <v>24</v>
       </c>
       <c r="F37" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G37" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>82</v>
       </c>
       <c r="H37" s="9" t="n">
         <v>5</v>
@@ -2402,7 +2405,7 @@
         <v>46309</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C38" s="10" t="s">
         <v>50</v>
@@ -2414,10 +2417,10 @@
         <v>24</v>
       </c>
       <c r="F38" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G38" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="G38" s="11" t="s">
-        <v>82</v>
       </c>
       <c r="H38" s="9" t="n">
         <v>1</v>
@@ -2438,7 +2441,7 @@
         <v>46309</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>56</v>
@@ -2450,10 +2453,10 @@
         <v>29</v>
       </c>
       <c r="F39" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G39" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>84</v>
       </c>
       <c r="H39" s="9" t="n">
         <v>5</v>
@@ -2474,7 +2477,7 @@
         <v>46309</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C40" s="10" t="s">
         <v>59</v>
@@ -2486,10 +2489,10 @@
         <v>29</v>
       </c>
       <c r="F40" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="G40" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="G40" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="H40" s="9" t="n">
         <v>1</v>
@@ -2510,10 +2513,10 @@
         <v>46309</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>23</v>
@@ -2546,10 +2549,10 @@
         <v>46309</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>34</v>
@@ -2558,10 +2561,10 @@
         <v>35</v>
       </c>
       <c r="F42" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="G42" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="G42" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="H42" s="9" t="n">
         <v>1</v>
@@ -2582,10 +2585,10 @@
         <v>46309</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>16</v>
@@ -2594,10 +2597,10 @@
         <v>38</v>
       </c>
       <c r="F43" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G43" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>86</v>
       </c>
       <c r="H43" s="9" t="n">
         <v>6</v>
@@ -2618,10 +2621,10 @@
         <v>46309</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>23</v>
@@ -2630,10 +2633,10 @@
         <v>38</v>
       </c>
       <c r="F44" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G44" s="11" t="s">
         <v>85</v>
-      </c>
-      <c r="G44" s="11" t="s">
-        <v>86</v>
       </c>
       <c r="H44" s="9" t="n">
         <v>1</v>
@@ -2654,7 +2657,7 @@
         <v>46310</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>43</v>
@@ -2666,10 +2669,10 @@
         <v>17</v>
       </c>
       <c r="F45" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G45" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>89</v>
       </c>
       <c r="H45" s="9" t="n">
         <v>1</v>
@@ -2690,7 +2693,7 @@
         <v>46310</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>46</v>
@@ -2702,10 +2705,10 @@
         <v>17</v>
       </c>
       <c r="F46" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="G46" s="11" t="s">
         <v>88</v>
-      </c>
-      <c r="G46" s="11" t="s">
-        <v>89</v>
       </c>
       <c r="H46" s="9" t="n">
         <v>1</v>
@@ -2726,7 +2729,7 @@
         <v>46310</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>47</v>
@@ -2738,10 +2741,10 @@
         <v>24</v>
       </c>
       <c r="F47" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G47" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>91</v>
       </c>
       <c r="H47" s="9" t="n">
         <v>5</v>
@@ -2762,7 +2765,7 @@
         <v>46310</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C48" s="10" t="s">
         <v>50</v>
@@ -2774,10 +2777,10 @@
         <v>24</v>
       </c>
       <c r="F48" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G48" s="11" t="s">
         <v>90</v>
-      </c>
-      <c r="G48" s="11" t="s">
-        <v>91</v>
       </c>
       <c r="H48" s="9" t="n">
         <v>1</v>
@@ -2798,7 +2801,7 @@
         <v>46310</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>56</v>
@@ -2810,10 +2813,10 @@
         <v>29</v>
       </c>
       <c r="F49" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G49" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="H49" s="9" t="n">
         <v>5</v>
@@ -2834,7 +2837,7 @@
         <v>46310</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C50" s="10" t="s">
         <v>59</v>
@@ -2846,10 +2849,10 @@
         <v>29</v>
       </c>
       <c r="F50" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="G50" s="11" t="s">
         <v>92</v>
-      </c>
-      <c r="G50" s="11" t="s">
-        <v>93</v>
       </c>
       <c r="H50" s="9" t="n">
         <v>1</v>
@@ -2870,10 +2873,10 @@
         <v>46310</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D51" s="15" t="s">
         <v>52</v>
@@ -2882,10 +2885,10 @@
         <v>35</v>
       </c>
       <c r="F51" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G51" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>96</v>
       </c>
       <c r="H51" s="9" t="n">
         <v>1</v>
@@ -2906,10 +2909,10 @@
         <v>46310</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D52" s="12" t="s">
         <v>23</v>
@@ -2918,10 +2921,10 @@
         <v>35</v>
       </c>
       <c r="F52" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="G52" s="11" t="s">
         <v>95</v>
-      </c>
-      <c r="G52" s="11" t="s">
-        <v>96</v>
       </c>
       <c r="H52" s="9" t="n">
         <v>1</v>
@@ -2942,10 +2945,10 @@
         <v>46310</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D53" s="14" t="s">
         <v>34</v>
@@ -2954,10 +2957,10 @@
         <v>35</v>
       </c>
       <c r="F53" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G53" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="H53" s="9" t="n">
         <v>1</v>
@@ -2978,10 +2981,10 @@
         <v>46310</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>16</v>
@@ -2990,10 +2993,10 @@
         <v>38</v>
       </c>
       <c r="F54" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="G54" s="11" t="s">
         <v>98</v>
-      </c>
-      <c r="G54" s="11" t="s">
-        <v>99</v>
       </c>
       <c r="H54" s="9" t="n">
         <v>5</v>
@@ -3014,10 +3017,10 @@
         <v>46310</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D55" s="12" t="s">
         <v>23</v>
@@ -3026,10 +3029,10 @@
         <v>38</v>
       </c>
       <c r="F55" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G55" s="5" t="s">
         <v>98</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>99</v>
       </c>
       <c r="H55" s="9" t="n">
         <v>1</v>
@@ -3050,7 +3053,7 @@
         <v>46311</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C56" s="10" t="s">
         <v>43</v>
@@ -3062,10 +3065,10 @@
         <v>17</v>
       </c>
       <c r="F56" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="G56" s="11" t="s">
         <v>101</v>
-      </c>
-      <c r="G56" s="11" t="s">
-        <v>102</v>
       </c>
       <c r="H56" s="9" t="n">
         <v>1</v>
@@ -3086,7 +3089,7 @@
         <v>46311</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>46</v>
@@ -3098,10 +3101,10 @@
         <v>17</v>
       </c>
       <c r="F57" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G57" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="G57" s="5" t="s">
-        <v>102</v>
       </c>
       <c r="H57" s="9" t="n">
         <v>1</v>
@@ -3122,7 +3125,7 @@
         <v>46311</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C58" s="10" t="s">
         <v>47</v>
@@ -3134,10 +3137,10 @@
         <v>24</v>
       </c>
       <c r="F58" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G58" s="11" t="s">
         <v>103</v>
-      </c>
-      <c r="G58" s="11" t="s">
-        <v>104</v>
       </c>
       <c r="H58" s="9" t="n">
         <v>1</v>
@@ -3158,7 +3161,7 @@
         <v>46311</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>50</v>
@@ -3170,10 +3173,10 @@
         <v>24</v>
       </c>
       <c r="F59" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="G59" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="G59" s="5" t="s">
-        <v>104</v>
       </c>
       <c r="H59" s="9" t="n">
         <v>1</v>
@@ -3194,10 +3197,10 @@
         <v>46311</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>16</v>
@@ -3206,10 +3209,10 @@
         <v>29</v>
       </c>
       <c r="F60" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="G60" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="G60" s="11" t="s">
-        <v>107</v>
       </c>
       <c r="H60" s="9" t="n">
         <v>1</v>
@@ -3230,10 +3233,10 @@
         <v>46311</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D61" s="12" t="s">
         <v>23</v>
@@ -3242,10 +3245,10 @@
         <v>29</v>
       </c>
       <c r="F61" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="G61" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="H61" s="9" t="n">
         <v>1</v>
@@ -3266,10 +3269,10 @@
         <v>46311</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>16</v>
@@ -3278,10 +3281,10 @@
         <v>38</v>
       </c>
       <c r="F62" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="G62" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="G62" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="H62" s="9" t="n">
         <v>1</v>
@@ -3302,10 +3305,10 @@
         <v>46311</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" s="12" t="s">
         <v>23</v>
@@ -3314,10 +3317,10 @@
         <v>38</v>
       </c>
       <c r="F63" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G63" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="G63" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="H63" s="9" t="n">
         <v>1</v>
@@ -3338,10 +3341,10 @@
         <v>46311</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D64" s="14" t="s">
         <v>34</v>
@@ -3350,10 +3353,10 @@
         <v>35</v>
       </c>
       <c r="F64" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="G64" s="11" t="s">
         <v>101</v>
-      </c>
-      <c r="G64" s="11" t="s">
-        <v>102</v>
       </c>
       <c r="H64" s="9" t="n">
         <v>1</v>
@@ -3374,10 +3377,10 @@
         <v>46312</v>
       </c>
       <c r="B65" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C65" s="6" t="s">
         <v>114</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>115</v>
       </c>
       <c r="D65" s="7" t="s">
         <v>16</v>
@@ -3386,10 +3389,10 @@
         <v>17</v>
       </c>
       <c r="F65" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="G65" s="5" t="s">
         <v>116</v>
-      </c>
-      <c r="G65" s="5" t="s">
-        <v>117</v>
       </c>
       <c r="H65" s="9" t="n">
         <v>1</v>
@@ -3410,10 +3413,10 @@
         <v>46312</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D66" s="12" t="s">
         <v>23</v>
@@ -3422,10 +3425,10 @@
         <v>17</v>
       </c>
       <c r="F66" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="G66" s="11" t="s">
         <v>116</v>
-      </c>
-      <c r="G66" s="11" t="s">
-        <v>117</v>
       </c>
       <c r="H66" s="9" t="n">
         <v>1</v>
@@ -3446,7 +3449,7 @@
         <v>46312</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>22</v>
@@ -3458,10 +3461,10 @@
         <v>24</v>
       </c>
       <c r="F67" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="G67" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="G67" s="5" t="s">
-        <v>120</v>
       </c>
       <c r="H67" s="9" t="n">
         <v>1</v>
@@ -3482,7 +3485,7 @@
         <v>46312</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C68" s="10" t="s">
         <v>27</v>
@@ -3494,10 +3497,10 @@
         <v>24</v>
       </c>
       <c r="F68" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="G68" s="11" t="s">
         <v>119</v>
-      </c>
-      <c r="G68" s="11" t="s">
-        <v>120</v>
       </c>
       <c r="H68" s="9" t="n">
         <v>1</v>
@@ -3518,10 +3521,10 @@
         <v>46312</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D69" s="7" t="s">
         <v>16</v>
@@ -3530,10 +3533,10 @@
         <v>29</v>
       </c>
       <c r="F69" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="G69" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="G69" s="5" t="s">
-        <v>123</v>
       </c>
       <c r="H69" s="9" t="n">
         <v>1</v>
@@ -3554,10 +3557,10 @@
         <v>46312</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>23</v>
@@ -3566,10 +3569,10 @@
         <v>29</v>
       </c>
       <c r="F70" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="G70" s="11" t="s">
         <v>122</v>
-      </c>
-      <c r="G70" s="11" t="s">
-        <v>123</v>
       </c>
       <c r="H70" s="9" t="n">
         <v>1</v>
@@ -3590,10 +3593,10 @@
         <v>46312</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>34</v>
@@ -3602,10 +3605,10 @@
         <v>35</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="H71" s="9" t="n">
         <v>1</v>
@@ -3626,10 +3629,10 @@
         <v>46312</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>16</v>
@@ -3638,10 +3641,10 @@
         <v>38</v>
       </c>
       <c r="F72" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G72" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H72" s="9" t="n">
         <v>1</v>
@@ -3662,10 +3665,10 @@
         <v>46312</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D73" s="12" t="s">
         <v>23</v>
@@ -3674,10 +3677,10 @@
         <v>38</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H73" s="9" t="n">
         <v>1</v>
@@ -3710,10 +3713,10 @@
         <v>17</v>
       </c>
       <c r="F74" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H74" s="9" t="n">
         <v>5</v>
@@ -3746,10 +3749,10 @@
         <v>17</v>
       </c>
       <c r="F75" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H75" s="9" t="n">
         <v>1</v>
@@ -3782,10 +3785,10 @@
         <v>24</v>
       </c>
       <c r="F76" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H76" s="9" t="n">
         <v>5</v>
@@ -3818,10 +3821,10 @@
         <v>24</v>
       </c>
       <c r="F77" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G77" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H77" s="9" t="n">
         <v>1</v>
@@ -3854,10 +3857,10 @@
         <v>29</v>
       </c>
       <c r="F78" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H78" s="9" t="n">
         <v>5</v>
@@ -3890,10 +3893,10 @@
         <v>29</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H79" s="9" t="n">
         <v>1</v>
@@ -3926,10 +3929,10 @@
         <v>35</v>
       </c>
       <c r="F80" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G80" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H80" s="9" t="n">
         <v>1</v>
@@ -3962,10 +3965,10 @@
         <v>38</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H81" s="9" t="n">
         <v>5</v>
@@ -3998,10 +4001,10 @@
         <v>38</v>
       </c>
       <c r="F82" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G82" s="11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H82" s="9" t="n">
         <v>1</v>
@@ -4034,10 +4037,10 @@
         <v>24</v>
       </c>
       <c r="F83" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H83" s="9" t="n">
         <v>4</v>
@@ -4070,10 +4073,10 @@
         <v>24</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G84" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H84" s="9" t="n">
         <v>1</v>
@@ -4089,12 +4092,84 @@
       </c>
       <c r="L84" s="11"/>
     </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="4" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F85" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="H85" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I85" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J85" s="9" t="n">
+        <v>1644</v>
+      </c>
+      <c r="K85" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="L85" s="5"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="4" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C86" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D86" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E86" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F86" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G86" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="H86" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I86" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="J86" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="L86" s="11"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L84"/>
+  <autoFilter ref="A4:L86"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
-  <conditionalFormatting sqref="K5:K84">
+  <conditionalFormatting sqref="K5:K86">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yayınlandı"</formula>
     </cfRule>
@@ -4103,7 +4178,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" error="Listeden seç: Bekliyor, Yayınlandı, Atlandı" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K84" type="list">
+    <dataValidation allowBlank="false" error="Listeden seç: Bekliyor, Yayınlandı, Atlandı" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K86" type="list">
       <formula1>"Bekliyor,Yayınlandı,Atlandı"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4124,7 +4199,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -4139,17 +4214,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4157,16 +4232,16 @@
         <v>5</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4174,16 +4249,16 @@
         <v>16</v>
       </c>
       <c r="B6" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A6)</f>
-        <v>33</v>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$86,A6)</f>
+        <v>34</v>
       </c>
       <c r="C6" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A6,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$86,A6,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D6" s="20" t="n">
         <f aca="false">B6-C6</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" s="21" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
@@ -4195,16 +4270,16 @@
         <v>23</v>
       </c>
       <c r="B7" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A7)</f>
-        <v>37</v>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$86,A7)</f>
+        <v>38</v>
       </c>
       <c r="C7" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A7,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$86,A7,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">B7-C7</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7" s="21" t="n">
         <f aca="false">IF(B7=0,0,C7/B7)</f>
@@ -4216,11 +4291,11 @@
         <v>34</v>
       </c>
       <c r="B8" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A8)</f>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$86,A8)</f>
         <v>8</v>
       </c>
       <c r="C8" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A8,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$86,A8,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D8" s="20" t="n">
@@ -4237,11 +4312,11 @@
         <v>52</v>
       </c>
       <c r="B9" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$D$5:$D$84,A9)</f>
+        <f aca="false">COUNTIF(Plan!$D$5:$D$86,A9)</f>
         <v>2</v>
       </c>
       <c r="C9" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$D$5:$D$84,A9,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$D$5:$D$86,A9,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D9" s="20" t="n">
@@ -4255,11 +4330,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B10" s="26" t="n">
         <f aca="false">SUM(B6:B9)</f>
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C10" s="26" t="n">
         <f aca="false">SUM(C6:C9)</f>
@@ -4267,7 +4342,7 @@
       </c>
       <c r="D10" s="26" t="n">
         <f aca="false">SUM(D6:D9)</f>
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E10" s="27" t="n">
         <f aca="false">IF(B10=0,0,C10/B10)</f>
@@ -4276,7 +4351,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4287,25 +4362,25 @@
         <v>3</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4316,19 +4391,19 @@
         <v>14</v>
       </c>
       <c r="C15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A15,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A15,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A15,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A15,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G15" s="20" t="n">
@@ -4336,7 +4411,7 @@
         <v>9</v>
       </c>
       <c r="H15" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A15,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A15,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I15" s="21" t="n">
@@ -4352,19 +4427,19 @@
         <v>42</v>
       </c>
       <c r="C16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A16,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A16,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A16,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A16,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>1</v>
       </c>
       <c r="G16" s="20" t="n">
@@ -4372,7 +4447,7 @@
         <v>11</v>
       </c>
       <c r="H16" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A16,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A16,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I16" s="21" t="n">
@@ -4388,19 +4463,19 @@
         <v>65</v>
       </c>
       <c r="C17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A17,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A17,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A17,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A17,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G17" s="20" t="n">
@@ -4408,7 +4483,7 @@
         <v>10</v>
       </c>
       <c r="H17" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A17,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A17,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I17" s="21" t="n">
@@ -4421,22 +4496,22 @@
         <v>46309</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A18,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A18,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A18,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A18,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G18" s="20" t="n">
@@ -4444,7 +4519,7 @@
         <v>10</v>
       </c>
       <c r="H18" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A18,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A18,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I18" s="21" t="n">
@@ -4457,22 +4532,22 @@
         <v>46310</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A19,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A19,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>5</v>
       </c>
       <c r="E19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A19,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A19,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>1</v>
       </c>
       <c r="G19" s="20" t="n">
@@ -4480,7 +4555,7 @@
         <v>11</v>
       </c>
       <c r="H19" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A19,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A19,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I19" s="21" t="n">
@@ -4493,22 +4568,22 @@
         <v>46311</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A20,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A20,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A20,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A20,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G20" s="20" t="n">
@@ -4516,7 +4591,7 @@
         <v>9</v>
       </c>
       <c r="H20" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A20,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A20,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I20" s="21" t="n">
@@ -4529,22 +4604,22 @@
         <v>46312</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A21,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A21,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A21,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A21,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G21" s="20" t="n">
@@ -4552,7 +4627,7 @@
         <v>9</v>
       </c>
       <c r="H21" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A21,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A21,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I21" s="21" t="n">
@@ -4568,19 +4643,19 @@
         <v>14</v>
       </c>
       <c r="C22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A22,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>4</v>
       </c>
       <c r="D22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A22,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>4</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A22,Plan!$D$5:$D$86,"REELS")</f>
         <v>1</v>
       </c>
       <c r="F22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A22,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G22" s="20" t="n">
@@ -4588,7 +4663,7 @@
         <v>9</v>
       </c>
       <c r="H22" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A22,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A22,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I22" s="21" t="n">
@@ -4604,19 +4679,19 @@
         <v>42</v>
       </c>
       <c r="C23" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"GÖNDERİ")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A23,Plan!$D$5:$D$86,"GÖNDERİ")</f>
         <v>1</v>
       </c>
       <c r="D23" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"HİKAYE")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A23,Plan!$D$5:$D$86,"HİKAYE")</f>
         <v>1</v>
       </c>
       <c r="E23" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"REELS")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A23,Plan!$D$5:$D$86,"REELS")</f>
         <v>0</v>
       </c>
       <c r="F23" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$D$5:$D$84,"KAMPANYA")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A23,Plan!$D$5:$D$86,"KAMPANYA")</f>
         <v>0</v>
       </c>
       <c r="G23" s="20" t="n">
@@ -4624,7 +4699,7 @@
         <v>2</v>
       </c>
       <c r="H23" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$84,$A23,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A23,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="I23" s="21" t="n">
@@ -4633,122 +4708,158 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25" t="s">
-        <v>146</v>
-      </c>
-      <c r="C24" s="26" t="n">
-        <f aca="false">SUM(C15:C23)</f>
-        <v>33</v>
-      </c>
-      <c r="D24" s="26" t="n">
-        <f aca="false">SUM(D15:D23)</f>
-        <v>37</v>
-      </c>
-      <c r="E24" s="26" t="n">
-        <f aca="false">SUM(E15:E23)</f>
+      <c r="A24" s="28" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A24,Plan!$D$5:$D$86,"GÖNDERİ")</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A24,Plan!$D$5:$D$86,"HİKAYE")</f>
+        <v>1</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A24,Plan!$D$5:$D$86,"REELS")</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A24,Plan!$D$5:$D$86,"KAMPANYA")</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="20" t="n">
+        <f aca="false">SUM(C24:F24)</f>
+        <v>2</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A24,Plan!$K$5:$K$86,"Yayınlandı")</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="21" t="n">
+        <f aca="false">IF(G24=0,0,H24/G24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25" s="26" t="n">
+        <f aca="false">SUM(C15:C24)</f>
+        <v>34</v>
+      </c>
+      <c r="D25" s="26" t="n">
+        <f aca="false">SUM(D15:D24)</f>
+        <v>38</v>
+      </c>
+      <c r="E25" s="26" t="n">
+        <f aca="false">SUM(E15:E24)</f>
         <v>8</v>
       </c>
-      <c r="F24" s="26" t="n">
-        <f aca="false">SUM(F15:F23)</f>
+      <c r="F25" s="26" t="n">
+        <f aca="false">SUM(F15:F24)</f>
         <v>2</v>
       </c>
-      <c r="G24" s="26" t="n">
-        <f aca="false">SUM(G15:G23)</f>
-        <v>80</v>
-      </c>
-      <c r="H24" s="26" t="n">
-        <f aca="false">SUM(H15:H23)</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <f aca="false">IF(G24=0,0,H24/G24)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>153</v>
+      <c r="G25" s="26" t="n">
+        <f aca="false">SUM(G15:G24)</f>
+        <v>82</v>
+      </c>
+      <c r="H25" s="26" t="n">
+        <f aca="false">SUM(H15:H24)</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <f aca="false">IF(G25=0,0,H25/G25)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="17" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="C28" s="18" t="s">
+      <c r="B29" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="D28" s="18" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="B29" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A29)</f>
-        <v>16</v>
-      </c>
-      <c r="C29" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A29,Plan!$K$5:$K$84,"Yayınlandı")</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A29,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A29,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
-        <v>1425</v>
+      <c r="C29" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="29" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B30" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A30)</f>
+        <f aca="false">COUNTIF(Plan!$E$5:$E$86,A30)</f>
         <v>18</v>
       </c>
       <c r="C30" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A30,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$86,A30,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D30" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A30,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A30,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
-        <v>1168</v>
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$86,Plan!$E$5:$E$86,A30,Plan!$D$5:$D$86,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$86,A30,Plan!$D$5:$D$86,"GÖNDERİ"),0),0)</f>
+        <v>1266</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="29" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B31" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A31)</f>
-        <v>16</v>
+        <f aca="false">COUNTIF(Plan!$E$5:$E$86,A31)</f>
+        <v>18</v>
       </c>
       <c r="C31" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A31,Plan!$K$5:$K$84,"Yayınlandı")</f>
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$86,A31,Plan!$K$5:$K$86,"Yayınlandı")</f>
         <v>0</v>
       </c>
       <c r="D31" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A31,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A31,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
-        <v>1508</v>
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$86,Plan!$E$5:$E$86,A31,Plan!$D$5:$D$86,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$86,A31,Plan!$D$5:$D$86,"GÖNDERİ"),0),0)</f>
+        <v>1168</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="20" t="n">
+        <f aca="false">COUNTIF(Plan!$E$5:$E$86,A32)</f>
+        <v>16</v>
+      </c>
+      <c r="C32" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$86,A32,Plan!$K$5:$K$86,"Yayınlandı")</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="20" t="n">
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$86,Plan!$E$5:$E$86,A32,Plan!$D$5:$D$86,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$86,A32,Plan!$D$5:$D$86,"GÖNDERİ"),0),0)</f>
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="20" t="n">
-        <f aca="false">COUNTIF(Plan!$E$5:$E$84,A32)</f>
+      <c r="B33" s="20" t="n">
+        <f aca="false">COUNTIF(Plan!$E$5:$E$86,A33)</f>
         <v>16</v>
       </c>
-      <c r="C32" s="20" t="n">
-        <f aca="false">COUNTIFS(Plan!$E$5:$E$84,A32,Plan!$K$5:$K$84,"Yayınlandı")</f>
-        <v>0</v>
-      </c>
-      <c r="D32" s="20" t="n">
-        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$84,Plan!$E$5:$E$84,A32,Plan!$D$5:$D$84,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$84,A32,Plan!$D$5:$D$84,"GÖNDERİ"),0),0)</f>
+      <c r="C33" s="20" t="n">
+        <f aca="false">COUNTIFS(Plan!$E$5:$E$86,A33,Plan!$K$5:$K$86,"Yayınlandı")</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$86,Plan!$E$5:$E$86,A33,Plan!$D$5:$D$86,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$86,A33,Plan!$D$5:$D$86,"GÖNDERİ"),0),0)</f>
         <v>1286</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dosyalar yenilendi — liste, paket sayfası, Excel
- metin.md'lerde '## Gönderi metni' başlığı eksikti; iki gönderinin
  metni pakette boş görünüyordu (biri yarın 12:38'de çıkacaktı)
- paket.py rehber gönderilerinin başlığını rehber.json'dan okuyor
- 13 Ekim 08:12 artık filament ayar rehberi

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DAKoXHyqFjWGSzqcjwTyja
</commit_message>
<xml_diff>
--- a/yayin-plani.xlsx
+++ b/yayin-plani.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="157">
   <si>
     <t xml:space="preserve">YAYIN PLANI · 11-18 Ekim 2026</t>
   </si>
@@ -222,6 +222,9 @@
   </si>
   <si>
     <t xml:space="preserve">Salı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FİLAMENT AYAR REHBERİ</t>
   </si>
   <si>
     <t xml:space="preserve">2026-10-21-filament-rehberi</t>
@@ -1952,7 +1955,7 @@
         <v>66</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H25" s="9" t="n">
         <v>1</v>
@@ -1961,7 +1964,7 @@
         <v>20</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>0</v>
+        <v>1385</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>21</v>
@@ -1988,7 +1991,7 @@
         <v>66</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H26" s="9" t="n">
         <v>1</v>
@@ -2021,10 +2024,10 @@
         <v>24</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H27" s="9" t="n">
         <v>4</v>
@@ -2033,7 +2036,7 @@
         <v>20</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>0</v>
+        <v>1410</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>21</v>
@@ -2057,10 +2060,10 @@
         <v>24</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H28" s="9" t="n">
         <v>1</v>
@@ -2093,10 +2096,10 @@
         <v>29</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H29" s="9" t="n">
         <v>5</v>
@@ -2129,10 +2132,10 @@
         <v>29</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H30" s="9" t="n">
         <v>1</v>
@@ -2156,7 +2159,7 @@
         <v>65</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>23</v>
@@ -2192,7 +2195,7 @@
         <v>65</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>34</v>
@@ -2201,10 +2204,10 @@
         <v>35</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H32" s="9" t="n">
         <v>1</v>
@@ -2228,7 +2231,7 @@
         <v>65</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>16</v>
@@ -2237,10 +2240,10 @@
         <v>38</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H33" s="9" t="n">
         <v>4</v>
@@ -2264,7 +2267,7 @@
         <v>65</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>23</v>
@@ -2273,10 +2276,10 @@
         <v>38</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H34" s="9" t="n">
         <v>1</v>
@@ -2297,7 +2300,7 @@
         <v>46309</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>43</v>
@@ -2309,10 +2312,10 @@
         <v>17</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H35" s="9" t="n">
         <v>4</v>
@@ -2333,7 +2336,7 @@
         <v>46309</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C36" s="10" t="s">
         <v>46</v>
@@ -2345,10 +2348,10 @@
         <v>17</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H36" s="9" t="n">
         <v>1</v>
@@ -2369,7 +2372,7 @@
         <v>46309</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>47</v>
@@ -2381,10 +2384,10 @@
         <v>24</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H37" s="9" t="n">
         <v>5</v>
@@ -2405,7 +2408,7 @@
         <v>46309</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C38" s="10" t="s">
         <v>50</v>
@@ -2417,10 +2420,10 @@
         <v>24</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H38" s="9" t="n">
         <v>1</v>
@@ -2441,7 +2444,7 @@
         <v>46309</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>56</v>
@@ -2453,10 +2456,10 @@
         <v>29</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H39" s="9" t="n">
         <v>5</v>
@@ -2477,7 +2480,7 @@
         <v>46309</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C40" s="10" t="s">
         <v>59</v>
@@ -2489,10 +2492,10 @@
         <v>29</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H40" s="9" t="n">
         <v>1</v>
@@ -2513,10 +2516,10 @@
         <v>46309</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>23</v>
@@ -2549,10 +2552,10 @@
         <v>46309</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>34</v>
@@ -2561,10 +2564,10 @@
         <v>35</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H42" s="9" t="n">
         <v>1</v>
@@ -2585,10 +2588,10 @@
         <v>46309</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>16</v>
@@ -2597,10 +2600,10 @@
         <v>38</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H43" s="9" t="n">
         <v>6</v>
@@ -2621,10 +2624,10 @@
         <v>46309</v>
       </c>
       <c r="B44" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>76</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>23</v>
@@ -2633,10 +2636,10 @@
         <v>38</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H44" s="9" t="n">
         <v>1</v>
@@ -2657,7 +2660,7 @@
         <v>46310</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>43</v>
@@ -2669,10 +2672,10 @@
         <v>17</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H45" s="9" t="n">
         <v>1</v>
@@ -2693,7 +2696,7 @@
         <v>46310</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>46</v>
@@ -2705,10 +2708,10 @@
         <v>17</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G46" s="11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H46" s="9" t="n">
         <v>1</v>
@@ -2729,7 +2732,7 @@
         <v>46310</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>47</v>
@@ -2741,10 +2744,10 @@
         <v>24</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H47" s="9" t="n">
         <v>5</v>
@@ -2765,7 +2768,7 @@
         <v>46310</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C48" s="10" t="s">
         <v>50</v>
@@ -2777,10 +2780,10 @@
         <v>24</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H48" s="9" t="n">
         <v>1</v>
@@ -2801,7 +2804,7 @@
         <v>46310</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>56</v>
@@ -2813,10 +2816,10 @@
         <v>29</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H49" s="9" t="n">
         <v>5</v>
@@ -2837,7 +2840,7 @@
         <v>46310</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C50" s="10" t="s">
         <v>59</v>
@@ -2849,10 +2852,10 @@
         <v>29</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G50" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H50" s="9" t="n">
         <v>1</v>
@@ -2873,10 +2876,10 @@
         <v>46310</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D51" s="15" t="s">
         <v>52</v>
@@ -2885,10 +2888,10 @@
         <v>35</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H51" s="9" t="n">
         <v>1</v>
@@ -2909,10 +2912,10 @@
         <v>46310</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D52" s="12" t="s">
         <v>23</v>
@@ -2921,10 +2924,10 @@
         <v>35</v>
       </c>
       <c r="F52" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G52" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H52" s="9" t="n">
         <v>1</v>
@@ -2945,10 +2948,10 @@
         <v>46310</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D53" s="14" t="s">
         <v>34</v>
@@ -2957,10 +2960,10 @@
         <v>35</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H53" s="9" t="n">
         <v>1</v>
@@ -2981,10 +2984,10 @@
         <v>46310</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>16</v>
@@ -2993,10 +2996,10 @@
         <v>38</v>
       </c>
       <c r="F54" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G54" s="11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H54" s="9" t="n">
         <v>5</v>
@@ -3017,10 +3020,10 @@
         <v>46310</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D55" s="12" t="s">
         <v>23</v>
@@ -3029,10 +3032,10 @@
         <v>38</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H55" s="9" t="n">
         <v>1</v>
@@ -3053,7 +3056,7 @@
         <v>46311</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C56" s="10" t="s">
         <v>43</v>
@@ -3065,10 +3068,10 @@
         <v>17</v>
       </c>
       <c r="F56" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H56" s="9" t="n">
         <v>1</v>
@@ -3089,7 +3092,7 @@
         <v>46311</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>46</v>
@@ -3101,10 +3104,10 @@
         <v>17</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H57" s="9" t="n">
         <v>1</v>
@@ -3125,7 +3128,7 @@
         <v>46311</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C58" s="10" t="s">
         <v>47</v>
@@ -3137,10 +3140,10 @@
         <v>24</v>
       </c>
       <c r="F58" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H58" s="9" t="n">
         <v>1</v>
@@ -3161,7 +3164,7 @@
         <v>46311</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>50</v>
@@ -3173,10 +3176,10 @@
         <v>24</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H59" s="9" t="n">
         <v>1</v>
@@ -3197,10 +3200,10 @@
         <v>46311</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>16</v>
@@ -3209,10 +3212,10 @@
         <v>29</v>
       </c>
       <c r="F60" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H60" s="9" t="n">
         <v>1</v>
@@ -3233,10 +3236,10 @@
         <v>46311</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D61" s="12" t="s">
         <v>23</v>
@@ -3245,10 +3248,10 @@
         <v>29</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H61" s="9" t="n">
         <v>1</v>
@@ -3269,10 +3272,10 @@
         <v>46311</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>16</v>
@@ -3281,10 +3284,10 @@
         <v>38</v>
       </c>
       <c r="F62" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G62" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H62" s="9" t="n">
         <v>1</v>
@@ -3305,10 +3308,10 @@
         <v>46311</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D63" s="12" t="s">
         <v>23</v>
@@ -3317,10 +3320,10 @@
         <v>38</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H63" s="9" t="n">
         <v>1</v>
@@ -3341,10 +3344,10 @@
         <v>46311</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D64" s="14" t="s">
         <v>34</v>
@@ -3353,10 +3356,10 @@
         <v>35</v>
       </c>
       <c r="F64" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G64" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H64" s="9" t="n">
         <v>1</v>
@@ -3377,10 +3380,10 @@
         <v>46312</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D65" s="7" t="s">
         <v>16</v>
@@ -3389,10 +3392,10 @@
         <v>17</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H65" s="9" t="n">
         <v>1</v>
@@ -3413,10 +3416,10 @@
         <v>46312</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D66" s="12" t="s">
         <v>23</v>
@@ -3425,10 +3428,10 @@
         <v>17</v>
       </c>
       <c r="F66" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G66" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H66" s="9" t="n">
         <v>1</v>
@@ -3449,7 +3452,7 @@
         <v>46312</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>22</v>
@@ -3461,10 +3464,10 @@
         <v>24</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G67" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H67" s="9" t="n">
         <v>1</v>
@@ -3485,7 +3488,7 @@
         <v>46312</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C68" s="10" t="s">
         <v>27</v>
@@ -3497,10 +3500,10 @@
         <v>24</v>
       </c>
       <c r="F68" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H68" s="9" t="n">
         <v>1</v>
@@ -3521,10 +3524,10 @@
         <v>46312</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D69" s="7" t="s">
         <v>16</v>
@@ -3533,10 +3536,10 @@
         <v>29</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H69" s="9" t="n">
         <v>1</v>
@@ -3557,10 +3560,10 @@
         <v>46312</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>23</v>
@@ -3569,10 +3572,10 @@
         <v>29</v>
       </c>
       <c r="F70" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H70" s="9" t="n">
         <v>1</v>
@@ -3593,10 +3596,10 @@
         <v>46312</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>34</v>
@@ -3605,10 +3608,10 @@
         <v>35</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H71" s="9" t="n">
         <v>1</v>
@@ -3629,10 +3632,10 @@
         <v>46312</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>16</v>
@@ -3641,10 +3644,10 @@
         <v>38</v>
       </c>
       <c r="F72" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G72" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H72" s="9" t="n">
         <v>1</v>
@@ -3665,10 +3668,10 @@
         <v>46312</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D73" s="12" t="s">
         <v>23</v>
@@ -3677,10 +3680,10 @@
         <v>38</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H73" s="9" t="n">
         <v>1</v>
@@ -3713,10 +3716,10 @@
         <v>17</v>
       </c>
       <c r="F74" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H74" s="9" t="n">
         <v>5</v>
@@ -3749,10 +3752,10 @@
         <v>17</v>
       </c>
       <c r="F75" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H75" s="9" t="n">
         <v>1</v>
@@ -3785,10 +3788,10 @@
         <v>24</v>
       </c>
       <c r="F76" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H76" s="9" t="n">
         <v>5</v>
@@ -3821,10 +3824,10 @@
         <v>24</v>
       </c>
       <c r="F77" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G77" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H77" s="9" t="n">
         <v>1</v>
@@ -3857,10 +3860,10 @@
         <v>29</v>
       </c>
       <c r="F78" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H78" s="9" t="n">
         <v>5</v>
@@ -3893,10 +3896,10 @@
         <v>29</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H79" s="9" t="n">
         <v>1</v>
@@ -3929,10 +3932,10 @@
         <v>35</v>
       </c>
       <c r="F80" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G80" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H80" s="9" t="n">
         <v>1</v>
@@ -3965,10 +3968,10 @@
         <v>38</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H81" s="9" t="n">
         <v>5</v>
@@ -4001,10 +4004,10 @@
         <v>38</v>
       </c>
       <c r="F82" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G82" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H82" s="9" t="n">
         <v>1</v>
@@ -4037,10 +4040,10 @@
         <v>24</v>
       </c>
       <c r="F83" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H83" s="9" t="n">
         <v>4</v>
@@ -4073,10 +4076,10 @@
         <v>24</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G84" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H84" s="9" t="n">
         <v>1</v>
@@ -4109,10 +4112,10 @@
         <v>17</v>
       </c>
       <c r="F85" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G85" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H85" s="9" t="n">
         <v>1</v>
@@ -4145,10 +4148,10 @@
         <v>17</v>
       </c>
       <c r="F86" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G86" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H86" s="9" t="n">
         <v>1</v>
@@ -4214,17 +4217,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4232,16 +4235,16 @@
         <v>5</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4330,7 +4333,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B10" s="26" t="n">
         <f aca="false">SUM(B6:B9)</f>
@@ -4351,7 +4354,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4362,25 +4365,25 @@
         <v>3</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4496,7 +4499,7 @@
         <v>46309</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C18" s="20" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A18,Plan!$D$5:$D$86,"GÖNDERİ")</f>
@@ -4532,7 +4535,7 @@
         <v>46310</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C19" s="20" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A19,Plan!$D$5:$D$86,"GÖNDERİ")</f>
@@ -4568,7 +4571,7 @@
         <v>46311</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C20" s="20" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A20,Plan!$D$5:$D$86,"GÖNDERİ")</f>
@@ -4604,7 +4607,7 @@
         <v>46312</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" s="20" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$86,$A21,Plan!$D$5:$D$86,"GÖNDERİ")</f>
@@ -4745,7 +4748,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="25" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C25" s="26" t="n">
         <f aca="false">SUM(C15:C24)</f>
@@ -4778,7 +4781,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4786,13 +4789,13 @@
         <v>6</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4809,7 +4812,7 @@
       </c>
       <c r="D30" s="20" t="n">
         <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$86,Plan!$E$5:$E$86,A30,Plan!$D$5:$D$86,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$86,A30,Plan!$D$5:$D$86,"GÖNDERİ"),0),0)</f>
-        <v>1266</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4826,7 +4829,7 @@
       </c>
       <c r="D31" s="20" t="n">
         <f aca="false">IFERROR(ROUND(SUMIFS(Plan!$J$5:$J$86,Plan!$E$5:$E$86,A31,Plan!$D$5:$D$86,"GÖNDERİ")/COUNTIFS(Plan!$E$5:$E$86,A31,Plan!$D$5:$D$86,"GÖNDERİ"),0),0)</f>
-        <v>1168</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>